<commit_message>
Fixed sign error for tax rate in forecast section
</commit_message>
<xml_diff>
--- a/1. List_ManualData.xlsx
+++ b/1. List_ManualData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1461D4F-715B-7E4C-94DE-6FD1AAC4E1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A8B628-4F78-7947-B144-0AB70DAABA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="100" windowWidth="25440" windowHeight="13540" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -636,7 +636,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="5">
-        <v>4.3999999999999997E-2</v>
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>